<commit_message>
Fase 4: cierre de resultados 2026-08-12
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,6 +527,162 @@
         <v>0</v>
       </c>
       <c r="L2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>FC Cincinnati vs Atlas</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FC Cincinnati</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Minnesota United FC vs Atlante</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Minnesota United FC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F4" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bolívar vs São Paulo</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F5" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -543,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -590,6 +746,25 @@
       </c>
       <c r="E2" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-13
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -685,6 +685,110 @@
       <c r="L5" t="inlineStr">
         <is>
           <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Toluca vs FC Dallas</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Toluca</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="F6" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Palmeiras vs Cerro Porteño</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Palmeiras</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="F7" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>5</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -699,7 +803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -765,6 +869,25 @@
       </c>
       <c r="E3" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -778,7 +901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -808,6 +931,111 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-14
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -803,7 +803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -888,6 +888,22 @@
       </c>
       <c r="E4" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-15
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -789,6 +789,266 @@
       <c r="L7" t="inlineStr">
         <is>
           <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Wolverhampton Wanderers vs Blackburn Rovers</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Wolverhampton Wanderers</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="F8" t="n">
+        <v>51</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Sporting CP vs Vitória de Guimaraes</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="F9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Galatasaray vs Çorum FK</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Galatasaray</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="F10" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Real Sociedad II vs Castellón</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Castellón</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="F11" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Telstar vs Sparta Rotterdam</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Telstar</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F12" t="n">
+        <v>81.5</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>si</t>
         </is>
       </c>
     </row>
@@ -803,7 +1063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -904,6 +1164,25 @@
       </c>
       <c r="E5" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>40</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-16
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1047,6 +1047,214 @@
         <v>0</v>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Fluminense vs Palmeiras</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Palmeiras</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="F13" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>São Paulo vs Coritiba</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Coritiba</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F14" t="n">
+        <v>71.3</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Atlante vs Toluca</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Toluca</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F15" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>2</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Orlando City SC vs FC Cincinnati</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Orlando City SC</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F16" t="n">
+        <v>66.5</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>3</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1063,7 +1271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1183,6 +1391,25 @@
       </c>
       <c r="E6" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1196,7 +1423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1331,6 +1558,90 @@
         <v>0</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-17
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -1271,7 +1271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1410,6 +1410,22 @@
       </c>
       <c r="E7" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-18
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1255,6 +1255,318 @@
         <v>1</v>
       </c>
       <c r="L16" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Almería vs Eldense</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Almería</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="F17" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>4</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Casa Pia vs Benfica</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Benfica</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="F18" t="n">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0-7</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>4</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Cardiff City vs Wrexham</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Cardiff City</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="F19" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>4</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Deportivo vs Elche</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Deportivo</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="F20" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Internacional vs Remo</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Remo</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="F21" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Lanús vs Independiente</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Lanús</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F22" t="n">
+        <v>72</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>4</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1271,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1426,6 +1738,25 @@
       </c>
       <c r="E8" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1439,7 +1770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1658,6 +1989,153 @@
         <v>0</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-19
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1567,6 +1567,110 @@
         <v>0</v>
       </c>
       <c r="L22" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia vs Fluminense</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="F23" t="n">
+        <v>67</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>4</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>São Paulo vs Bolívar</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="F24" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>5</v>
+      </c>
+      <c r="J24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" t="n">
+        <v>1</v>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1583,7 +1687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1757,6 +1861,25 @@
       </c>
       <c r="E9" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1770,7 +1893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2136,6 +2259,111 @@
         <v>0</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-20
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -1687,7 +1687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1880,6 +1880,22 @@
       </c>
       <c r="E10" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-21
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -1687,7 +1687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1895,6 +1895,22 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-22
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1671,6 +1671,58 @@
         <v>1</v>
       </c>
       <c r="L24" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Erzurum BB vs Galatasaray</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Galatasaray</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="F25" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>1</v>
+      </c>
+      <c r="L25" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1687,7 +1739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1912,6 +1964,25 @@
       </c>
       <c r="E12" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1925,7 +1996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2396,6 +2467,48 @@
         <v>100</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-23
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1723,6 +1723,318 @@
         <v>1</v>
       </c>
       <c r="L25" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Albacete vs Real Sociedad II</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Albacete</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="F26" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>1</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Sporting CP vs Alverca</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="F27" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Wrexham vs Watford</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Wrexham</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="F28" t="n">
+        <v>78.5</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Sparta Rotterdam vs FC Utrecht</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>FC Utrecht</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="F29" t="n">
+        <v>70.09999999999999</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>5</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Fluminense vs Remo</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Remo</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="F30" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>2</v>
+      </c>
+      <c r="J30" t="n">
+        <v>2</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Vancouver Whitecaps vs FC Dallas</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Vancouver Whitecaps</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="F31" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>3</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>1</v>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -1739,7 +2051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1983,6 +2295,25 @@
       </c>
       <c r="E13" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="E14" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1996,7 +2327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2509,6 +2840,69 @@
         <v>0</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>7</v>
+      </c>
+      <c r="D26" t="n">
+        <v>4</v>
+      </c>
+      <c r="E26" t="n">
+        <v>57.1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-24
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2035,6 +2035,58 @@
         <v>1</v>
       </c>
       <c r="L31" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Elche vs Barcelona</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="F32" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0-5</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>3</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -2051,7 +2103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2314,6 +2366,25 @@
       </c>
       <c r="E14" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>100</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2327,7 +2398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2903,6 +2974,69 @@
         <v>0</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-25
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2087,6 +2087,110 @@
         <v>0</v>
       </c>
       <c r="L32" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Málaga vs Deportivo</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Málaga</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="F33" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>2</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Lanús vs Argentinos Juniors</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Lanús</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="F34" t="n">
+        <v>55</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -2103,7 +2207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2385,6 +2489,25 @@
       </c>
       <c r="E15" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2398,7 +2521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3037,6 +3160,48 @@
         <v>0</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-26
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -2207,7 +2207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2508,6 +2508,22 @@
       </c>
       <c r="E16" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-27
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -2207,7 +2207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2523,6 +2523,22 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-29
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2295,6 +2295,162 @@
         <v>0</v>
       </c>
       <c r="L36" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Wrexham vs Birmingham City</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Birmingham City</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="F37" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>2</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Rio Ave vs Sporting CP</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="F38" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
+        <v>2</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Racing Santander vs Elche</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F39" t="n">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
+        <v>2</v>
+      </c>
+      <c r="L39" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -2311,7 +2467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2663,6 +2819,25 @@
       </c>
       <c r="E19" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-30
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2451,6 +2451,318 @@
         <v>2</v>
       </c>
       <c r="L39" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Galatasaray vs Goztepe</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Galatasaray</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F40" t="n">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>6</v>
+      </c>
+      <c r="J40" t="n">
+        <v>2</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Cardiff City vs Sheffield United</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Cardiff City</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="F41" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Watford vs West Ham United</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>West Ham United</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="F42" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" t="n">
+        <v>1</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Albacete vs Real Oviedo</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Albacete</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="F43" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
+        <v>1</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Excelsior vs Sparta Rotterdam</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Excelsior</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="F44" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>2</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Sporting Kansas City vs Vancouver Whitecaps</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Sporting Kansas City</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="F45" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>1</v>
+      </c>
+      <c r="L45" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -2467,7 +2779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2838,6 +3150,25 @@
       </c>
       <c r="E20" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2851,7 +3182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3532,6 +3863,69 @@
         <v>0</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>4</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-08-31
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2763,6 +2763,1462 @@
         <v>1</v>
       </c>
       <c r="L45" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Sunderland vs Fulham</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Sunderland</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F46" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Manchester United vs Ipswich Town</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Manchester United</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="F47" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Real Madrid vs Málaga</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="F48" t="n">
+        <v>45</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Mallorca vs Ceuta</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Mallorca</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="F49" t="n">
+        <v>38.8</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>1</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>SC Freiburg vs Werder Bremen</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>SC Freiburg</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="F50" t="n">
+        <v>65.40000000000001</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>FC Augsburg vs Schalke 04</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Schalke 04</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="F51" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Paris FC vs Nice</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Paris FC</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F52" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Feyenoord Rotterdam vs ADO Den Haag</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Feyenoord Rotterdam</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="F53" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Willem II vs Heerenveen</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Willem II</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="F54" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Telstar vs Ajax Amsterdam</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Telstar</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="F55" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Argentinos Juniors vs Aldosivi</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Argentinos Juniors</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="F56" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>7</v>
+      </c>
+      <c r="J56" t="n">
+        <v>1</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Toluca vs FC Juarez</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Toluca</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F57" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Chelsea vs Brighton &amp; Hove Albion</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Brighton &amp; Hove Albion</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="F58" t="n">
+        <v>38</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Leeds United vs Brentford</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Leeds United</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="F59" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Deportivo vs Valencia</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Deportivo</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="F60" t="n">
+        <v>43</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" t="n">
+        <v>2</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Cagliari vs Internazionale</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="F61" t="n">
+        <v>39</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>5</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Stade Rennais vs Le Mans</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Le Mans</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="F62" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>AS Monaco vs Marseille</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Marseille</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="F63" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>FC Utrecht vs PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="F64" t="n">
+        <v>68.09999999999999</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>1-6</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" t="n">
+        <v>1</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>SC Cambuur vs FC Twente</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>SC Cambuur</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="F65" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>1</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>FC Famalicao vs Gil Vicente</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>FC Famalicao</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="F66" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>1</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>KAA Gent vs Club Brugge</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Club Brugge</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F67" t="n">
+        <v>89.40000000000001</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Union St.-Gilloise vs Anderlecht</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Union St.-Gilloise</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="F68" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>KVC Westerlo vs Zulte-Waregem</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Zulte-Waregem</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="F69" t="n">
+        <v>73.90000000000001</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Aris vs OFI Crete</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Aris</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="F70" t="n">
+        <v>76</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Asteras Tripoli vs Olympiacos</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Asteras Tripoli</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="F71" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0</v>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Kifisia vs AEK Athens</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Kifisia</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="F72" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>1</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" t="n">
+        <v>0</v>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Athletico-PR vs Fluminense</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Athletico-PR</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="F73" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" t="n">
+        <v>3</v>
+      </c>
+      <c r="L73" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -2779,7 +4235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3169,6 +4625,25 @@
       </c>
       <c r="E21" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>28</v>
+      </c>
+      <c r="C22" t="n">
+        <v>12</v>
+      </c>
+      <c r="D22" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="E22" t="n">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -3182,7 +4657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3926,6 +5401,132 @@
         <v>25</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>8</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-03
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4583,6 +4583,58 @@
         <v>2</v>
       </c>
       <c r="L80" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Millwall vs Wrexham</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Millwall</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F81" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0</v>
+      </c>
+      <c r="K81" t="n">
+        <v>3</v>
+      </c>
+      <c r="L81" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -4599,7 +4651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5046,6 +5098,25 @@
       </c>
       <c r="E24" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5059,7 +5130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6055,6 +6126,27 @@
         <v>25</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-05
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4687,6 +4687,214 @@
         <v>0</v>
       </c>
       <c r="L82" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Real Betis vs Real Madrid</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="F83" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>3</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K83" t="n">
+        <v>1</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain vs AS Monaco</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="F84" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>8</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" t="n">
+        <v>1</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Sparta Rotterdam vs PEC Zwolle</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Sparta Rotterdam</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="F85" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>3</v>
+      </c>
+      <c r="J85" t="n">
+        <v>3</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Lommel SK vs Club Brugge</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Club Brugge</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="F86" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" t="n">
+        <v>1</v>
+      </c>
+      <c r="L86" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -4703,7 +4911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5188,6 +5396,25 @@
       </c>
       <c r="E26" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="n">
+        <v>25</v>
+      </c>
+      <c r="E27" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -5201,7 +5428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6218,6 +6445,111 @@
         <v>0</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>6</v>
+      </c>
+      <c r="D50" t="n">
+        <v>2</v>
+      </c>
+      <c r="E50" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-06
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4895,6 +4895,994 @@
         <v>1</v>
       </c>
       <c r="L86" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Preston North End vs Blackburn Rovers</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Preston North End</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="F87" t="n">
+        <v>51</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>0</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" t="n">
+        <v>1</v>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>West Ham United vs Derby County</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>West Ham United</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="F88" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>0</v>
+      </c>
+      <c r="J88" t="n">
+        <v>2</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Villarreal vs Deportivo</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="F89" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>5</v>
+      </c>
+      <c r="J89" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" t="n">
+        <v>3</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Schalke 04 vs Bayern Munich</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="F90" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>3</v>
+      </c>
+      <c r="J90" t="n">
+        <v>1</v>
+      </c>
+      <c r="K90" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>NEC Nijmegen vs Feyenoord Rotterdam</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Feyenoord Rotterdam</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="F91" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
+        <v>1</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Maritimo vs Benfica</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Benfica</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="F92" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>1</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0</v>
+      </c>
+      <c r="K92" t="n">
+        <v>2</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Sporting CP vs C.D. Nacional</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="F93" t="n">
+        <v>61</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>7</v>
+      </c>
+      <c r="J93" t="n">
+        <v>3</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Volos NFC vs Olympiacos</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Olympiacos</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F94" t="n">
+        <v>81.2</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>0</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0</v>
+      </c>
+      <c r="K94" t="n">
+        <v>1</v>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>FC Dallas vs Sporting Kansas City</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>FC Dallas</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="F95" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>0</v>
+      </c>
+      <c r="J95" t="n">
+        <v>2</v>
+      </c>
+      <c r="K95" t="n">
+        <v>1</v>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Vancouver Whitecaps vs St. Louis CITY SC</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Vancouver Whitecaps</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="F96" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>0</v>
+      </c>
+      <c r="J96" t="n">
+        <v>2</v>
+      </c>
+      <c r="K96" t="n">
+        <v>0</v>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Fulham vs Crystal Palace</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Fulham</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="F97" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>0</v>
+      </c>
+      <c r="J97" t="n">
+        <v>1</v>
+      </c>
+      <c r="K97" t="n">
+        <v>0</v>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>West Bromwich Albion vs Watford</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>West Bromwich Albion</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="F98" t="n">
+        <v>87.09999999999999</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>0</v>
+      </c>
+      <c r="J98" t="n">
+        <v>0</v>
+      </c>
+      <c r="K98" t="n">
+        <v>3</v>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Swansea City vs Wrexham</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Swansea City</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F99" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>1</v>
+      </c>
+      <c r="J99" t="n">
+        <v>1</v>
+      </c>
+      <c r="K99" t="n">
+        <v>4</v>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Rayo Vallecano vs Racing Santander</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="F100" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>2</v>
+      </c>
+      <c r="J100" t="n">
+        <v>1</v>
+      </c>
+      <c r="K100" t="n">
+        <v>1</v>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Werder Bremen vs RB Leipzig</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>RB Leipzig</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="F101" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>0</v>
+      </c>
+      <c r="J101" t="n">
+        <v>1</v>
+      </c>
+      <c r="K101" t="n">
+        <v>0</v>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Nice vs Le Mans</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Le Mans</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="F102" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>3</v>
+      </c>
+      <c r="J102" t="n">
+        <v>1</v>
+      </c>
+      <c r="K102" t="n">
+        <v>1</v>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Ajax Amsterdam vs PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="F103" t="n">
+        <v>67</v>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>3</v>
+      </c>
+      <c r="J103" t="n">
+        <v>1</v>
+      </c>
+      <c r="K103" t="n">
+        <v>1</v>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Willem II vs Excelsior</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Excelsior</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="F104" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>6</v>
+      </c>
+      <c r="J104" t="n">
+        <v>1</v>
+      </c>
+      <c r="K104" t="n">
+        <v>1</v>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>AEK Athens vs Aris</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Aris</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="F105" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>1</v>
+      </c>
+      <c r="J105" t="n">
+        <v>1</v>
+      </c>
+      <c r="K105" t="n">
+        <v>1</v>
+      </c>
+      <c r="L105" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -4911,7 +5899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5415,6 +6403,25 @@
       </c>
       <c r="E27" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>19</v>
+      </c>
+      <c r="C28" t="n">
+        <v>9</v>
+      </c>
+      <c r="D28" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="E28" t="n">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -5428,7 +6435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6550,6 +7557,174 @@
         <v>0</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>14</v>
+      </c>
+      <c r="D54" t="n">
+        <v>2</v>
+      </c>
+      <c r="E54" t="n">
+        <v>14.3</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>5</v>
+      </c>
+      <c r="D55" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>3</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>6</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-07
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5883,6 +5883,578 @@
         <v>1</v>
       </c>
       <c r="L105" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Everton vs Manchester United</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Everton</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="F106" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>0</v>
+      </c>
+      <c r="J106" t="n">
+        <v>0</v>
+      </c>
+      <c r="K106" t="n">
+        <v>1</v>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Arsenal vs Chelsea</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="F107" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>0</v>
+      </c>
+      <c r="J107" t="n">
+        <v>0</v>
+      </c>
+      <c r="K107" t="n">
+        <v>1</v>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Valencia vs Barcelona</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="F108" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>0-5</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>0</v>
+      </c>
+      <c r="J108" t="n">
+        <v>1</v>
+      </c>
+      <c r="K108" t="n">
+        <v>3</v>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Heerenveen vs AZ Alkmaar</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Heerenveen</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="F109" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>0</v>
+      </c>
+      <c r="J109" t="n">
+        <v>1</v>
+      </c>
+      <c r="K109" t="n">
+        <v>0</v>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>ADO Den Haag vs Fortuna Sittard</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>ADO Den Haag</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="F110" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>0</v>
+      </c>
+      <c r="J110" t="n">
+        <v>1</v>
+      </c>
+      <c r="K110" t="n">
+        <v>0</v>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>OFI Crete vs Kifisia</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>OFI Crete</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="F111" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>0</v>
+      </c>
+      <c r="J111" t="n">
+        <v>1</v>
+      </c>
+      <c r="K111" t="n">
+        <v>1</v>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Remo vs Flamengo</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Remo</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="F112" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>4</v>
+      </c>
+      <c r="J112" t="n">
+        <v>2</v>
+      </c>
+      <c r="K112" t="n">
+        <v>0</v>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Málaga vs Levante</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Málaga</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="F113" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>3</v>
+      </c>
+      <c r="J113" t="n">
+        <v>2</v>
+      </c>
+      <c r="K113" t="n">
+        <v>0</v>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Telstar vs SC Cambuur</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Telstar</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="F114" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>0</v>
+      </c>
+      <c r="J114" t="n">
+        <v>2</v>
+      </c>
+      <c r="K114" t="n">
+        <v>1</v>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Vitória de Guimaraes vs Casa Pia</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Vitória de Guimaraes</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="F115" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>3</v>
+      </c>
+      <c r="J115" t="n">
+        <v>2</v>
+      </c>
+      <c r="K115" t="n">
+        <v>1</v>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Cercle Brugge KSV vs KAA Gent</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Cercle Brugge KSV</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="F116" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>0</v>
+      </c>
+      <c r="J116" t="n">
+        <v>0</v>
+      </c>
+      <c r="K116" t="n">
+        <v>1</v>
+      </c>
+      <c r="L116" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -5899,7 +6471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6422,6 +6994,25 @@
       </c>
       <c r="E28" t="n">
         <v>19</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>11</v>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="E29" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -6435,7 +7026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7725,6 +8316,111 @@
         <v>0</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>6</v>
+      </c>
+      <c r="D62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>